<commit_message>
Cambios para ver resumen de insumos
</commit_message>
<xml_diff>
--- a/backend/app/reports/templates/plantilla_dashboard.xlsx
+++ b/backend/app/reports/templates/plantilla_dashboard.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/r06xd/Documents/Personal/proyecto_omar/agrostak-app/backend/app/reports/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E2F6476-1937-0E48-9EBA-76F267F7676A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{427287BB-E0C8-D046-80D3-DFB3F340A88A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11620" yWindow="5560" windowWidth="28040" windowHeight="17440" xr2:uid="{9550B607-3B25-2C4D-8F29-2F77220F3381}"/>
   </bookViews>
@@ -114,10 +114,10 @@
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
+      <c14:style val="103"/>
     </mc:Choice>
     <mc:Fallback>
-      <c:style val="2"/>
+      <c:style val="3"/>
     </mc:Fallback>
   </mc:AlternateContent>
   <c:chart>
@@ -154,10 +154,8 @@
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
       <c:layout/>
-      <c:barChart>
-        <c:barDir val="col"/>
-        <c:grouping val="clustered"/>
-        <c:varyColors val="0"/>
+      <c:doughnutChart>
+        <c:varyColors val="1"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
@@ -169,16 +167,79 @@
               </c:strCache>
             </c:strRef>
           </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent1"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:shade val="53000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:shade val="76000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="3"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:tint val="77000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="4"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:tint val="54000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
           <c:cat>
             <c:numRef>
               <c:f>datos!$A$5:$A$9</c:f>
@@ -210,119 +271,11 @@
           <c:showSerName val="0"/>
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
         </c:dLbls>
-        <c:gapWidth val="219"/>
-        <c:overlap val="-27"/>
-        <c:axId val="1170979760"/>
-        <c:axId val="1199682640"/>
-      </c:barChart>
-      <c:catAx>
-        <c:axId val="1170979760"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="15000"/>
-                <a:lumOff val="85000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-EC"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1199682640"/>
-        <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="1199682640"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-EC"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1170979760"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
-      </c:valAx>
+        <c:firstSliceAng val="0"/>
+        <c:holeSize val="50"/>
+      </c:doughnutChart>
       <c:spPr>
         <a:noFill/>
         <a:ln>
@@ -694,42 +647,8 @@
 </file>
 
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="withinLinear" id="14">
   <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
 </cs:colorStyle>
 </file>
 

</xml_diff>